<commit_message>
chore(electricidad): generic download button + 3-sheet summary Excel (Q1/Q2/Q3)
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mensual GWh" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1 Installed Capacity (MW)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2 Consumption (GWh)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3 Invoiced by Sector (GWh)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,13 +415,1380 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Hydro</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Thermal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>GEE</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Biomass</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Solar</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Wind</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Biogas</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B2" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-307.7</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-234.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B3" t="n">
+        <v>550</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-5.5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>545.7</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B4" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-13.8</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-3.600000000000001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B6" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-48.6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-39.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B7" t="n">
+        <v>79.09999999999999</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>107.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G8" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>61.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B9" t="n">
+        <v>218.9</v>
+      </c>
+      <c r="C9" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>359.6</v>
+      </c>
+      <c r="E9" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="I9" t="n">
+        <v>715.1999999999999</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B10" t="n">
+        <v>-14.8</v>
+      </c>
+      <c r="C10" t="n">
+        <v>228.5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>47</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>46.8</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>307.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B11" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>204.4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-1.1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>230</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B100"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Consumption_GWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Jan 2018</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2158.8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Feb 2018</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1848.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Mar 2018</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2078.4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Apr 2018</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2072.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>May 2018</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2090.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jun 2018</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1920.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jul 2018</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1935.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Aug 2018</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1954.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sep 2018</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1936.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Oct 2018</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1978.1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Nov 2018</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1962.9</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Dec 2018</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2065.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Jan 2019</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2214.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Feb 2019</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2146.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Mar 2019</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Apr 2019</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2274.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>May 2019</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>2330.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Jun 2019</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2179.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Jul 2019</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2160.9</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Aug 2019</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2195.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sep 2019</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>2112.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Oct 2019</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2101.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Nov 2019</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2202.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Dec 2019</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>2303.2</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jan 2020</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>2415.8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Feb 2020</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2259.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Mar 2020</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2183.1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Apr 2020</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2026.2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>May 2020</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2190.4</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Jun 2020</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>2185.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jul 2020</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>2207.7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Aug 2020</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2147.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Sep 2020</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2051.3</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Oct 2020</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>2182.6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Nov 2020</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>2058.4</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Dec 2020</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>2276.4</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Jan 2021</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2175.8</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Feb 2021</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>2028.4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Mar 2021</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>2448.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Apr 2021</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>2375.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>May 2021</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>2203.9</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Jun 2021</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>2076.6</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Jul 2021</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>2123.1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Aug 2021</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2156.9</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Sep 2021</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>2128</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Oct 2021</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>2245.8</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Nov 2021</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2163</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Dec 2021</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>2373.7</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Jan 2022</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>2296.2</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Feb 2022</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>2085.2</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Mar 2022</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>2439</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Apr 2022</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>2386.6</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>May 2022</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>2369.3</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Jun 2022</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>2119</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Jul 2022</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>2230.9</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Aug 2022</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>2246.6</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Sep 2022</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>2258.1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Oct 2022</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>2272.8</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Nov 2022</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>2267.5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Dec 2022</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2481.9</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Jan 2023</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>2582</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Feb 2023</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2245</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Mar 2023</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>2543.7</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Apr 2023</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2492.6</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>May 2023</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>2769.1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Jun 2023</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2643.2</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Jul 2023</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2716.3</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Aug 2023</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2555.7</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Sep 2023</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>2489.4</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Oct 2023</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>2585.2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Nov 2023</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>2403.3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Dec 2023</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2513.7</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Jan 2024</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>2615.5</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Feb 2024</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2487.6</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Mar 2024</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>2757.3</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Apr 2024</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2556.3</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>May 2024</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2708.4</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Jun 2024</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2518.3</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Jul 2024</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2537</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Aug 2024</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2514.8</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Sep 2024</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>2286.8</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Oct 2024</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1975.5</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Nov 2024</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1853.5</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Dec 2024</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2355.2</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Jan 2025</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>2604.6</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Feb 2025</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2566.3</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Mar 2025</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>2849</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Apr 2025</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2774.5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>May 2025</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>2794.3</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>2573.7</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>2605.6</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Aug 2025</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>2592.2</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Sep 2025</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>2667.9</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Oct 2025</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>2802.6</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Nov 2025</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>2696.6</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Dec 2025</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>2828.5</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Jan 2026</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>2683.2</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Feb 2026</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>2606.8</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>3002.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Fecha</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">

</xml_diff>

<commit_message>
chore: ARCONEL update — data through May 2026
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1 Installed Capacity (MW)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2 Consumption (GWh)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3 Invoiced by Sector (GWh)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Q1 Installed Capacity (MW)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Q2 Consumption (GWh)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Q3 Invoiced by Sector (GWh)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B100"/>
+  <dimension ref="A1:B102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2683.2</v>
+        <v>2685.5</v>
       </c>
     </row>
     <row r="99">
@@ -1758,7 +1758,7 @@
         </is>
       </c>
       <c r="B99" t="n">
-        <v>2606.8</v>
+        <v>2609.1</v>
       </c>
     </row>
     <row r="100">
@@ -1768,7 +1768,27 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>3002.8</v>
+        <v>3010.2</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Apr 2026</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>2911.6</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>May 2026</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>3016.5</v>
       </c>
     </row>
   </sheetData>
@@ -1782,7 +1802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4002,19 +4022,63 @@
         </is>
       </c>
       <c r="B101" t="n">
-        <v>24.93087</v>
+        <v>143.805073</v>
       </c>
       <c r="C101" t="n">
-        <v>42.050904</v>
+        <v>434.091955</v>
       </c>
       <c r="D101" t="n">
-        <v>52.459198</v>
+        <v>586.932054</v>
       </c>
       <c r="E101" t="n">
-        <v>23.137308</v>
+        <v>290.062914</v>
       </c>
       <c r="F101" t="n">
-        <v>104.268904</v>
+        <v>901.131844</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>148.657828</v>
+      </c>
+      <c r="C102" t="n">
+        <v>438.592339</v>
+      </c>
+      <c r="D102" t="n">
+        <v>590.10272</v>
+      </c>
+      <c r="E102" t="n">
+        <v>309.826588</v>
+      </c>
+      <c r="F102" t="n">
+        <v>883.625599</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>12.80218</v>
+      </c>
+      <c r="C103" t="n">
+        <v>21.427225</v>
+      </c>
+      <c r="D103" t="n">
+        <v>24.662815</v>
+      </c>
+      <c r="E103" t="n">
+        <v>6.463591</v>
+      </c>
+      <c r="F103" t="n">
+        <v>41.41849</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: ARCONEL update — data through Jun 2026
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Q1 Installed Capacity (MW)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Q2 Consumption (GWh)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Q3 Invoiced by Sector (GWh)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1 Installed Capacity (MW)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2 Consumption (GWh)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3 Invoiced by Sector (GWh)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B102"/>
+  <dimension ref="A1:B103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="B98" t="n">
-        <v>2685.5</v>
+        <v>2685.6</v>
       </c>
     </row>
     <row r="99">
@@ -1788,7 +1788,17 @@
         </is>
       </c>
       <c r="B102" t="n">
-        <v>3016.5</v>
+        <v>3074.6</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>2985.4</v>
       </c>
     </row>
   </sheetData>
@@ -4066,19 +4076,19 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>12.80218</v>
+        <v>151.60361</v>
       </c>
       <c r="C103" t="n">
-        <v>21.427225</v>
+        <v>440.199396</v>
       </c>
       <c r="D103" t="n">
-        <v>24.662815</v>
+        <v>631.125211</v>
       </c>
       <c r="E103" t="n">
-        <v>6.463591</v>
+        <v>362.220161</v>
       </c>
       <c r="F103" t="n">
-        <v>41.41849</v>
+        <v>867.371383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: update electricidad dashboard
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:C103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,6 +780,11 @@
           <t>Consumption_GWh</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Trend (GWh)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -790,6 +795,9 @@
       <c r="B2" t="n">
         <v>2158.8</v>
       </c>
+      <c r="C2" t="n">
+        <v>1973.1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -800,6 +808,9 @@
       <c r="B3" t="n">
         <v>1848.8</v>
       </c>
+      <c r="C3" t="n">
+        <v>1980.6</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -810,6 +821,9 @@
       <c r="B4" t="n">
         <v>2078.4</v>
       </c>
+      <c r="C4" t="n">
+        <v>1988.2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -820,6 +834,9 @@
       <c r="B5" t="n">
         <v>2072.8</v>
       </c>
+      <c r="C5" t="n">
+        <v>1995.7</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -830,6 +847,9 @@
       <c r="B6" t="n">
         <v>2090.8</v>
       </c>
+      <c r="C6" t="n">
+        <v>2003.2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -840,6 +860,9 @@
       <c r="B7" t="n">
         <v>1920.9</v>
       </c>
+      <c r="C7" t="n">
+        <v>2010.8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -850,6 +873,9 @@
       <c r="B8" t="n">
         <v>1935.5</v>
       </c>
+      <c r="C8" t="n">
+        <v>2018.3</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -860,6 +886,9 @@
       <c r="B9" t="n">
         <v>1954.2</v>
       </c>
+      <c r="C9" t="n">
+        <v>2025.8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -870,6 +899,9 @@
       <c r="B10" t="n">
         <v>1936.6</v>
       </c>
+      <c r="C10" t="n">
+        <v>2033.4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -880,6 +912,9 @@
       <c r="B11" t="n">
         <v>1978.1</v>
       </c>
+      <c r="C11" t="n">
+        <v>2040.9</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -890,6 +925,9 @@
       <c r="B12" t="n">
         <v>1962.9</v>
       </c>
+      <c r="C12" t="n">
+        <v>2048.4</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -900,6 +938,9 @@
       <c r="B13" t="n">
         <v>2065.3</v>
       </c>
+      <c r="C13" t="n">
+        <v>2056</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -910,6 +951,9 @@
       <c r="B14" t="n">
         <v>2214.6</v>
       </c>
+      <c r="C14" t="n">
+        <v>2063.5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -920,6 +964,9 @@
       <c r="B15" t="n">
         <v>2146.8</v>
       </c>
+      <c r="C15" t="n">
+        <v>2071</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -930,6 +977,9 @@
       <c r="B16" t="n">
         <v>2357</v>
       </c>
+      <c r="C16" t="n">
+        <v>2078.6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -940,6 +990,9 @@
       <c r="B17" t="n">
         <v>2274.1</v>
       </c>
+      <c r="C17" t="n">
+        <v>2086.1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -950,6 +1003,9 @@
       <c r="B18" t="n">
         <v>2330.3</v>
       </c>
+      <c r="C18" t="n">
+        <v>2093.6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -960,6 +1016,9 @@
       <c r="B19" t="n">
         <v>2179.6</v>
       </c>
+      <c r="C19" t="n">
+        <v>2101.1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -970,6 +1029,9 @@
       <c r="B20" t="n">
         <v>2160.9</v>
       </c>
+      <c r="C20" t="n">
+        <v>2108.7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -980,6 +1042,9 @@
       <c r="B21" t="n">
         <v>2195.7</v>
       </c>
+      <c r="C21" t="n">
+        <v>2116.2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -990,6 +1055,9 @@
       <c r="B22" t="n">
         <v>2112.2</v>
       </c>
+      <c r="C22" t="n">
+        <v>2123.7</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1000,6 +1068,9 @@
       <c r="B23" t="n">
         <v>2101.2</v>
       </c>
+      <c r="C23" t="n">
+        <v>2131.3</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1010,6 +1081,9 @@
       <c r="B24" t="n">
         <v>2202.4</v>
       </c>
+      <c r="C24" t="n">
+        <v>2138.8</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1020,6 +1094,9 @@
       <c r="B25" t="n">
         <v>2303.2</v>
       </c>
+      <c r="C25" t="n">
+        <v>2146.3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1030,6 +1107,9 @@
       <c r="B26" t="n">
         <v>2415.8</v>
       </c>
+      <c r="C26" t="n">
+        <v>2153.9</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1040,6 +1120,9 @@
       <c r="B27" t="n">
         <v>2259.1</v>
       </c>
+      <c r="C27" t="n">
+        <v>2161.4</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1050,6 +1133,9 @@
       <c r="B28" t="n">
         <v>2183.1</v>
       </c>
+      <c r="C28" t="n">
+        <v>2168.9</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1060,6 +1146,9 @@
       <c r="B29" t="n">
         <v>2026.2</v>
       </c>
+      <c r="C29" t="n">
+        <v>2176.5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1070,6 +1159,9 @@
       <c r="B30" t="n">
         <v>2190.4</v>
       </c>
+      <c r="C30" t="n">
+        <v>2184</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1080,6 +1172,9 @@
       <c r="B31" t="n">
         <v>2185.5</v>
       </c>
+      <c r="C31" t="n">
+        <v>2191.5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1090,6 +1185,9 @@
       <c r="B32" t="n">
         <v>2207.7</v>
       </c>
+      <c r="C32" t="n">
+        <v>2199.1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1100,6 +1198,9 @@
       <c r="B33" t="n">
         <v>2147.2</v>
       </c>
+      <c r="C33" t="n">
+        <v>2206.6</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1110,6 +1211,9 @@
       <c r="B34" t="n">
         <v>2051.3</v>
       </c>
+      <c r="C34" t="n">
+        <v>2214.1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1120,6 +1224,9 @@
       <c r="B35" t="n">
         <v>2182.6</v>
       </c>
+      <c r="C35" t="n">
+        <v>2221.7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1130,6 +1237,9 @@
       <c r="B36" t="n">
         <v>2058.4</v>
       </c>
+      <c r="C36" t="n">
+        <v>2229.2</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1140,6 +1250,9 @@
       <c r="B37" t="n">
         <v>2276.4</v>
       </c>
+      <c r="C37" t="n">
+        <v>2236.7</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1150,6 +1263,9 @@
       <c r="B38" t="n">
         <v>2175.8</v>
       </c>
+      <c r="C38" t="n">
+        <v>2244.3</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1160,6 +1276,9 @@
       <c r="B39" t="n">
         <v>2028.4</v>
       </c>
+      <c r="C39" t="n">
+        <v>2251.8</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1170,6 +1289,9 @@
       <c r="B40" t="n">
         <v>2448.4</v>
       </c>
+      <c r="C40" t="n">
+        <v>2259.3</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1180,6 +1302,9 @@
       <c r="B41" t="n">
         <v>2375.5</v>
       </c>
+      <c r="C41" t="n">
+        <v>2266.9</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1190,6 +1315,9 @@
       <c r="B42" t="n">
         <v>2203.9</v>
       </c>
+      <c r="C42" t="n">
+        <v>2274.4</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1200,6 +1328,9 @@
       <c r="B43" t="n">
         <v>2076.6</v>
       </c>
+      <c r="C43" t="n">
+        <v>2281.9</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1210,6 +1341,9 @@
       <c r="B44" t="n">
         <v>2123.1</v>
       </c>
+      <c r="C44" t="n">
+        <v>2289.5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1220,6 +1354,9 @@
       <c r="B45" t="n">
         <v>2156.9</v>
       </c>
+      <c r="C45" t="n">
+        <v>2297</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1230,6 +1367,9 @@
       <c r="B46" t="n">
         <v>2128</v>
       </c>
+      <c r="C46" t="n">
+        <v>2304.5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1240,6 +1380,9 @@
       <c r="B47" t="n">
         <v>2245.8</v>
       </c>
+      <c r="C47" t="n">
+        <v>2312.1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1250,6 +1393,9 @@
       <c r="B48" t="n">
         <v>2163</v>
       </c>
+      <c r="C48" t="n">
+        <v>2319.6</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1260,6 +1406,9 @@
       <c r="B49" t="n">
         <v>2373.7</v>
       </c>
+      <c r="C49" t="n">
+        <v>2327.1</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1270,6 +1419,9 @@
       <c r="B50" t="n">
         <v>2296.2</v>
       </c>
+      <c r="C50" t="n">
+        <v>2334.6</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1280,6 +1432,9 @@
       <c r="B51" t="n">
         <v>2085.2</v>
       </c>
+      <c r="C51" t="n">
+        <v>2342.2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1290,6 +1445,9 @@
       <c r="B52" t="n">
         <v>2439</v>
       </c>
+      <c r="C52" t="n">
+        <v>2349.7</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1300,6 +1458,9 @@
       <c r="B53" t="n">
         <v>2386.6</v>
       </c>
+      <c r="C53" t="n">
+        <v>2357.2</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1310,6 +1471,9 @@
       <c r="B54" t="n">
         <v>2369.3</v>
       </c>
+      <c r="C54" t="n">
+        <v>2364.8</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1320,6 +1484,9 @@
       <c r="B55" t="n">
         <v>2119</v>
       </c>
+      <c r="C55" t="n">
+        <v>2372.3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1330,6 +1497,9 @@
       <c r="B56" t="n">
         <v>2230.9</v>
       </c>
+      <c r="C56" t="n">
+        <v>2379.8</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1340,6 +1510,9 @@
       <c r="B57" t="n">
         <v>2246.6</v>
       </c>
+      <c r="C57" t="n">
+        <v>2387.4</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1350,6 +1523,9 @@
       <c r="B58" t="n">
         <v>2258.1</v>
       </c>
+      <c r="C58" t="n">
+        <v>2394.9</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1360,6 +1536,9 @@
       <c r="B59" t="n">
         <v>2272.8</v>
       </c>
+      <c r="C59" t="n">
+        <v>2402.4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1370,6 +1549,9 @@
       <c r="B60" t="n">
         <v>2267.5</v>
       </c>
+      <c r="C60" t="n">
+        <v>2410</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1380,6 +1562,9 @@
       <c r="B61" t="n">
         <v>2481.9</v>
       </c>
+      <c r="C61" t="n">
+        <v>2417.5</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1390,6 +1575,9 @@
       <c r="B62" t="n">
         <v>2582</v>
       </c>
+      <c r="C62" t="n">
+        <v>2425</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1400,6 +1588,9 @@
       <c r="B63" t="n">
         <v>2245</v>
       </c>
+      <c r="C63" t="n">
+        <v>2432.6</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1410,6 +1601,9 @@
       <c r="B64" t="n">
         <v>2543.7</v>
       </c>
+      <c r="C64" t="n">
+        <v>2440.1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1420,6 +1614,9 @@
       <c r="B65" t="n">
         <v>2492.6</v>
       </c>
+      <c r="C65" t="n">
+        <v>2447.6</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1430,6 +1627,9 @@
       <c r="B66" t="n">
         <v>2769.1</v>
       </c>
+      <c r="C66" t="n">
+        <v>2455.2</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1440,6 +1640,9 @@
       <c r="B67" t="n">
         <v>2643.2</v>
       </c>
+      <c r="C67" t="n">
+        <v>2462.7</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1450,6 +1653,9 @@
       <c r="B68" t="n">
         <v>2716.3</v>
       </c>
+      <c r="C68" t="n">
+        <v>2470.2</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1460,6 +1666,9 @@
       <c r="B69" t="n">
         <v>2555.7</v>
       </c>
+      <c r="C69" t="n">
+        <v>2477.8</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1470,6 +1679,9 @@
       <c r="B70" t="n">
         <v>2489.4</v>
       </c>
+      <c r="C70" t="n">
+        <v>2485.3</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1480,6 +1692,9 @@
       <c r="B71" t="n">
         <v>2585.2</v>
       </c>
+      <c r="C71" t="n">
+        <v>2492.8</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1490,6 +1705,9 @@
       <c r="B72" t="n">
         <v>2403.3</v>
       </c>
+      <c r="C72" t="n">
+        <v>2500.4</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1500,6 +1718,9 @@
       <c r="B73" t="n">
         <v>2513.7</v>
       </c>
+      <c r="C73" t="n">
+        <v>2507.9</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1510,6 +1731,9 @@
       <c r="B74" t="n">
         <v>2615.5</v>
       </c>
+      <c r="C74" t="n">
+        <v>2515.4</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1520,6 +1744,9 @@
       <c r="B75" t="n">
         <v>2487.6</v>
       </c>
+      <c r="C75" t="n">
+        <v>2523</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1530,6 +1757,9 @@
       <c r="B76" t="n">
         <v>2757.3</v>
       </c>
+      <c r="C76" t="n">
+        <v>2530.5</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1540,6 +1770,9 @@
       <c r="B77" t="n">
         <v>2556.3</v>
       </c>
+      <c r="C77" t="n">
+        <v>2538</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1550,6 +1783,9 @@
       <c r="B78" t="n">
         <v>2708.4</v>
       </c>
+      <c r="C78" t="n">
+        <v>2545.5</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1560,6 +1796,9 @@
       <c r="B79" t="n">
         <v>2518.3</v>
       </c>
+      <c r="C79" t="n">
+        <v>2553.1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1570,6 +1809,9 @@
       <c r="B80" t="n">
         <v>2537</v>
       </c>
+      <c r="C80" t="n">
+        <v>2560.6</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1580,6 +1822,9 @@
       <c r="B81" t="n">
         <v>2514.8</v>
       </c>
+      <c r="C81" t="n">
+        <v>2568.1</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1590,6 +1835,9 @@
       <c r="B82" t="n">
         <v>2286.8</v>
       </c>
+      <c r="C82" t="n">
+        <v>2575.7</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1600,6 +1848,9 @@
       <c r="B83" t="n">
         <v>1975.5</v>
       </c>
+      <c r="C83" t="n">
+        <v>2583.2</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1610,6 +1861,9 @@
       <c r="B84" t="n">
         <v>1853.5</v>
       </c>
+      <c r="C84" t="n">
+        <v>2590.7</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1620,6 +1874,9 @@
       <c r="B85" t="n">
         <v>2355.2</v>
       </c>
+      <c r="C85" t="n">
+        <v>2598.3</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1630,6 +1887,9 @@
       <c r="B86" t="n">
         <v>2604.6</v>
       </c>
+      <c r="C86" t="n">
+        <v>2605.8</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1640,6 +1900,9 @@
       <c r="B87" t="n">
         <v>2566.3</v>
       </c>
+      <c r="C87" t="n">
+        <v>2613.3</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1650,6 +1913,9 @@
       <c r="B88" t="n">
         <v>2849</v>
       </c>
+      <c r="C88" t="n">
+        <v>2620.9</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1660,6 +1926,9 @@
       <c r="B89" t="n">
         <v>2774.5</v>
       </c>
+      <c r="C89" t="n">
+        <v>2628.4</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1670,6 +1939,9 @@
       <c r="B90" t="n">
         <v>2794.3</v>
       </c>
+      <c r="C90" t="n">
+        <v>2635.9</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1680,6 +1952,9 @@
       <c r="B91" t="n">
         <v>2573.7</v>
       </c>
+      <c r="C91" t="n">
+        <v>2643.5</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1690,6 +1965,9 @@
       <c r="B92" t="n">
         <v>2605.6</v>
       </c>
+      <c r="C92" t="n">
+        <v>2651</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1700,6 +1978,9 @@
       <c r="B93" t="n">
         <v>2592.2</v>
       </c>
+      <c r="C93" t="n">
+        <v>2658.5</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1710,6 +1991,9 @@
       <c r="B94" t="n">
         <v>2667.9</v>
       </c>
+      <c r="C94" t="n">
+        <v>2666.1</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1720,6 +2004,9 @@
       <c r="B95" t="n">
         <v>2802.6</v>
       </c>
+      <c r="C95" t="n">
+        <v>2673.6</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1730,6 +2017,9 @@
       <c r="B96" t="n">
         <v>2696.6</v>
       </c>
+      <c r="C96" t="n">
+        <v>2681.1</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1740,6 +2030,9 @@
       <c r="B97" t="n">
         <v>2828.5</v>
       </c>
+      <c r="C97" t="n">
+        <v>2688.7</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1750,6 +2043,9 @@
       <c r="B98" t="n">
         <v>2685.6</v>
       </c>
+      <c r="C98" t="n">
+        <v>2696.2</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1760,6 +2056,9 @@
       <c r="B99" t="n">
         <v>2609.1</v>
       </c>
+      <c r="C99" t="n">
+        <v>2703.7</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1770,6 +2069,9 @@
       <c r="B100" t="n">
         <v>3010.2</v>
       </c>
+      <c r="C100" t="n">
+        <v>2711.3</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1780,6 +2082,9 @@
       <c r="B101" t="n">
         <v>2911.6</v>
       </c>
+      <c r="C101" t="n">
+        <v>2718.8</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1790,6 +2095,9 @@
       <c r="B102" t="n">
         <v>3074.6</v>
       </c>
+      <c r="C102" t="n">
+        <v>2726.3</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1799,6 +2107,9 @@
       </c>
       <c r="B103" t="n">
         <v>2985.4</v>
+      </c>
+      <c r="C103" t="n">
+        <v>2733.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: ARCONEL update — data through Jul 2026
</commit_message>
<xml_diff>
--- a/electricidad/facturacion_clientes_regulados_resumen.xlsx
+++ b/electricidad/facturacion_clientes_regulados_resumen.xlsx
@@ -766,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C103"/>
+  <dimension ref="A1:C104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,7 +796,7 @@
         <v>2158.8</v>
       </c>
       <c r="C2" t="n">
-        <v>1973.1</v>
+        <v>1963.3</v>
       </c>
     </row>
     <row r="3">
@@ -809,7 +809,7 @@
         <v>1848.8</v>
       </c>
       <c r="C3" t="n">
-        <v>1980.6</v>
+        <v>1971.2</v>
       </c>
     </row>
     <row r="4">
@@ -822,7 +822,7 @@
         <v>2078.4</v>
       </c>
       <c r="C4" t="n">
-        <v>1988.2</v>
+        <v>1979</v>
       </c>
     </row>
     <row r="5">
@@ -835,7 +835,7 @@
         <v>2072.8</v>
       </c>
       <c r="C5" t="n">
-        <v>1995.7</v>
+        <v>1986.8</v>
       </c>
     </row>
     <row r="6">
@@ -848,7 +848,7 @@
         <v>2090.8</v>
       </c>
       <c r="C6" t="n">
-        <v>2003.2</v>
+        <v>1994.6</v>
       </c>
     </row>
     <row r="7">
@@ -861,7 +861,7 @@
         <v>1920.9</v>
       </c>
       <c r="C7" t="n">
-        <v>2010.8</v>
+        <v>2002.4</v>
       </c>
     </row>
     <row r="8">
@@ -874,7 +874,7 @@
         <v>1935.5</v>
       </c>
       <c r="C8" t="n">
-        <v>2018.3</v>
+        <v>2010.3</v>
       </c>
     </row>
     <row r="9">
@@ -887,7 +887,7 @@
         <v>1954.2</v>
       </c>
       <c r="C9" t="n">
-        <v>2025.8</v>
+        <v>2018.1</v>
       </c>
     </row>
     <row r="10">
@@ -900,7 +900,7 @@
         <v>1936.6</v>
       </c>
       <c r="C10" t="n">
-        <v>2033.4</v>
+        <v>2025.9</v>
       </c>
     </row>
     <row r="11">
@@ -913,7 +913,7 @@
         <v>1978.1</v>
       </c>
       <c r="C11" t="n">
-        <v>2040.9</v>
+        <v>2033.7</v>
       </c>
     </row>
     <row r="12">
@@ -926,7 +926,7 @@
         <v>1962.9</v>
       </c>
       <c r="C12" t="n">
-        <v>2048.4</v>
+        <v>2041.6</v>
       </c>
     </row>
     <row r="13">
@@ -939,7 +939,7 @@
         <v>2065.3</v>
       </c>
       <c r="C13" t="n">
-        <v>2056</v>
+        <v>2049.4</v>
       </c>
     </row>
     <row r="14">
@@ -952,7 +952,7 @@
         <v>2214.6</v>
       </c>
       <c r="C14" t="n">
-        <v>2063.5</v>
+        <v>2057.2</v>
       </c>
     </row>
     <row r="15">
@@ -965,7 +965,7 @@
         <v>2146.8</v>
       </c>
       <c r="C15" t="n">
-        <v>2071</v>
+        <v>2065</v>
       </c>
     </row>
     <row r="16">
@@ -978,7 +978,7 @@
         <v>2357</v>
       </c>
       <c r="C16" t="n">
-        <v>2078.6</v>
+        <v>2072.8</v>
       </c>
     </row>
     <row r="17">
@@ -991,7 +991,7 @@
         <v>2274.1</v>
       </c>
       <c r="C17" t="n">
-        <v>2086.1</v>
+        <v>2080.7</v>
       </c>
     </row>
     <row r="18">
@@ -1004,7 +1004,7 @@
         <v>2330.3</v>
       </c>
       <c r="C18" t="n">
-        <v>2093.6</v>
+        <v>2088.5</v>
       </c>
     </row>
     <row r="19">
@@ -1017,7 +1017,7 @@
         <v>2179.6</v>
       </c>
       <c r="C19" t="n">
-        <v>2101.1</v>
+        <v>2096.3</v>
       </c>
     </row>
     <row r="20">
@@ -1030,7 +1030,7 @@
         <v>2160.9</v>
       </c>
       <c r="C20" t="n">
-        <v>2108.7</v>
+        <v>2104.1</v>
       </c>
     </row>
     <row r="21">
@@ -1043,7 +1043,7 @@
         <v>2195.7</v>
       </c>
       <c r="C21" t="n">
-        <v>2116.2</v>
+        <v>2112</v>
       </c>
     </row>
     <row r="22">
@@ -1056,7 +1056,7 @@
         <v>2112.2</v>
       </c>
       <c r="C22" t="n">
-        <v>2123.7</v>
+        <v>2119.8</v>
       </c>
     </row>
     <row r="23">
@@ -1069,7 +1069,7 @@
         <v>2101.2</v>
       </c>
       <c r="C23" t="n">
-        <v>2131.3</v>
+        <v>2127.6</v>
       </c>
     </row>
     <row r="24">
@@ -1082,7 +1082,7 @@
         <v>2202.4</v>
       </c>
       <c r="C24" t="n">
-        <v>2138.8</v>
+        <v>2135.4</v>
       </c>
     </row>
     <row r="25">
@@ -1095,7 +1095,7 @@
         <v>2303.2</v>
       </c>
       <c r="C25" t="n">
-        <v>2146.3</v>
+        <v>2143.3</v>
       </c>
     </row>
     <row r="26">
@@ -1108,7 +1108,7 @@
         <v>2415.8</v>
       </c>
       <c r="C26" t="n">
-        <v>2153.9</v>
+        <v>2151.1</v>
       </c>
     </row>
     <row r="27">
@@ -1121,7 +1121,7 @@
         <v>2259.1</v>
       </c>
       <c r="C27" t="n">
-        <v>2161.4</v>
+        <v>2158.9</v>
       </c>
     </row>
     <row r="28">
@@ -1134,7 +1134,7 @@
         <v>2183.1</v>
       </c>
       <c r="C28" t="n">
-        <v>2168.9</v>
+        <v>2166.7</v>
       </c>
     </row>
     <row r="29">
@@ -1147,7 +1147,7 @@
         <v>2026.2</v>
       </c>
       <c r="C29" t="n">
-        <v>2176.5</v>
+        <v>2174.5</v>
       </c>
     </row>
     <row r="30">
@@ -1160,7 +1160,7 @@
         <v>2190.4</v>
       </c>
       <c r="C30" t="n">
-        <v>2184</v>
+        <v>2182.4</v>
       </c>
     </row>
     <row r="31">
@@ -1173,7 +1173,7 @@
         <v>2185.5</v>
       </c>
       <c r="C31" t="n">
-        <v>2191.5</v>
+        <v>2190.2</v>
       </c>
     </row>
     <row r="32">
@@ -1186,7 +1186,7 @@
         <v>2207.7</v>
       </c>
       <c r="C32" t="n">
-        <v>2199.1</v>
+        <v>2198</v>
       </c>
     </row>
     <row r="33">
@@ -1199,7 +1199,7 @@
         <v>2147.2</v>
       </c>
       <c r="C33" t="n">
-        <v>2206.6</v>
+        <v>2205.8</v>
       </c>
     </row>
     <row r="34">
@@ -1212,7 +1212,7 @@
         <v>2051.3</v>
       </c>
       <c r="C34" t="n">
-        <v>2214.1</v>
+        <v>2213.7</v>
       </c>
     </row>
     <row r="35">
@@ -1225,7 +1225,7 @@
         <v>2182.6</v>
       </c>
       <c r="C35" t="n">
-        <v>2221.7</v>
+        <v>2221.5</v>
       </c>
     </row>
     <row r="36">
@@ -1238,7 +1238,7 @@
         <v>2058.4</v>
       </c>
       <c r="C36" t="n">
-        <v>2229.2</v>
+        <v>2229.3</v>
       </c>
     </row>
     <row r="37">
@@ -1251,7 +1251,7 @@
         <v>2276.4</v>
       </c>
       <c r="C37" t="n">
-        <v>2236.7</v>
+        <v>2237.1</v>
       </c>
     </row>
     <row r="38">
@@ -1264,7 +1264,7 @@
         <v>2175.8</v>
       </c>
       <c r="C38" t="n">
-        <v>2244.3</v>
+        <v>2244.9</v>
       </c>
     </row>
     <row r="39">
@@ -1277,7 +1277,7 @@
         <v>2028.4</v>
       </c>
       <c r="C39" t="n">
-        <v>2251.8</v>
+        <v>2252.8</v>
       </c>
     </row>
     <row r="40">
@@ -1290,7 +1290,7 @@
         <v>2448.4</v>
       </c>
       <c r="C40" t="n">
-        <v>2259.3</v>
+        <v>2260.6</v>
       </c>
     </row>
     <row r="41">
@@ -1303,7 +1303,7 @@
         <v>2375.5</v>
       </c>
       <c r="C41" t="n">
-        <v>2266.9</v>
+        <v>2268.4</v>
       </c>
     </row>
     <row r="42">
@@ -1316,7 +1316,7 @@
         <v>2203.9</v>
       </c>
       <c r="C42" t="n">
-        <v>2274.4</v>
+        <v>2276.2</v>
       </c>
     </row>
     <row r="43">
@@ -1329,7 +1329,7 @@
         <v>2076.6</v>
       </c>
       <c r="C43" t="n">
-        <v>2281.9</v>
+        <v>2284.1</v>
       </c>
     </row>
     <row r="44">
@@ -1342,7 +1342,7 @@
         <v>2123.1</v>
       </c>
       <c r="C44" t="n">
-        <v>2289.5</v>
+        <v>2291.9</v>
       </c>
     </row>
     <row r="45">
@@ -1355,7 +1355,7 @@
         <v>2156.9</v>
       </c>
       <c r="C45" t="n">
-        <v>2297</v>
+        <v>2299.7</v>
       </c>
     </row>
     <row r="46">
@@ -1368,7 +1368,7 @@
         <v>2128</v>
       </c>
       <c r="C46" t="n">
-        <v>2304.5</v>
+        <v>2307.5</v>
       </c>
     </row>
     <row r="47">
@@ -1381,7 +1381,7 @@
         <v>2245.8</v>
       </c>
       <c r="C47" t="n">
-        <v>2312.1</v>
+        <v>2315.4</v>
       </c>
     </row>
     <row r="48">
@@ -1394,7 +1394,7 @@
         <v>2163</v>
       </c>
       <c r="C48" t="n">
-        <v>2319.6</v>
+        <v>2323.2</v>
       </c>
     </row>
     <row r="49">
@@ -1407,7 +1407,7 @@
         <v>2373.7</v>
       </c>
       <c r="C49" t="n">
-        <v>2327.1</v>
+        <v>2331</v>
       </c>
     </row>
     <row r="50">
@@ -1420,7 +1420,7 @@
         <v>2296.2</v>
       </c>
       <c r="C50" t="n">
-        <v>2334.6</v>
+        <v>2338.8</v>
       </c>
     </row>
     <row r="51">
@@ -1433,7 +1433,7 @@
         <v>2085.2</v>
       </c>
       <c r="C51" t="n">
-        <v>2342.2</v>
+        <v>2346.6</v>
       </c>
     </row>
     <row r="52">
@@ -1446,7 +1446,7 @@
         <v>2439</v>
       </c>
       <c r="C52" t="n">
-        <v>2349.7</v>
+        <v>2354.5</v>
       </c>
     </row>
     <row r="53">
@@ -1459,7 +1459,7 @@
         <v>2386.6</v>
       </c>
       <c r="C53" t="n">
-        <v>2357.2</v>
+        <v>2362.3</v>
       </c>
     </row>
     <row r="54">
@@ -1472,7 +1472,7 @@
         <v>2369.3</v>
       </c>
       <c r="C54" t="n">
-        <v>2364.8</v>
+        <v>2370.1</v>
       </c>
     </row>
     <row r="55">
@@ -1485,7 +1485,7 @@
         <v>2119</v>
       </c>
       <c r="C55" t="n">
-        <v>2372.3</v>
+        <v>2377.9</v>
       </c>
     </row>
     <row r="56">
@@ -1498,7 +1498,7 @@
         <v>2230.9</v>
       </c>
       <c r="C56" t="n">
-        <v>2379.8</v>
+        <v>2385.8</v>
       </c>
     </row>
     <row r="57">
@@ -1511,7 +1511,7 @@
         <v>2246.6</v>
       </c>
       <c r="C57" t="n">
-        <v>2387.4</v>
+        <v>2393.6</v>
       </c>
     </row>
     <row r="58">
@@ -1524,7 +1524,7 @@
         <v>2258.1</v>
       </c>
       <c r="C58" t="n">
-        <v>2394.9</v>
+        <v>2401.4</v>
       </c>
     </row>
     <row r="59">
@@ -1537,7 +1537,7 @@
         <v>2272.8</v>
       </c>
       <c r="C59" t="n">
-        <v>2402.4</v>
+        <v>2409.2</v>
       </c>
     </row>
     <row r="60">
@@ -1550,7 +1550,7 @@
         <v>2267.5</v>
       </c>
       <c r="C60" t="n">
-        <v>2410</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="61">
@@ -1563,7 +1563,7 @@
         <v>2481.9</v>
       </c>
       <c r="C61" t="n">
-        <v>2417.5</v>
+        <v>2424.9</v>
       </c>
     </row>
     <row r="62">
@@ -1576,7 +1576,7 @@
         <v>2582</v>
       </c>
       <c r="C62" t="n">
-        <v>2425</v>
+        <v>2432.7</v>
       </c>
     </row>
     <row r="63">
@@ -1589,7 +1589,7 @@
         <v>2245</v>
       </c>
       <c r="C63" t="n">
-        <v>2432.6</v>
+        <v>2440.5</v>
       </c>
     </row>
     <row r="64">
@@ -1602,7 +1602,7 @@
         <v>2543.7</v>
       </c>
       <c r="C64" t="n">
-        <v>2440.1</v>
+        <v>2448.3</v>
       </c>
     </row>
     <row r="65">
@@ -1615,7 +1615,7 @@
         <v>2492.6</v>
       </c>
       <c r="C65" t="n">
-        <v>2447.6</v>
+        <v>2456.2</v>
       </c>
     </row>
     <row r="66">
@@ -1628,7 +1628,7 @@
         <v>2769.1</v>
       </c>
       <c r="C66" t="n">
-        <v>2455.2</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="67">
@@ -1641,7 +1641,7 @@
         <v>2643.2</v>
       </c>
       <c r="C67" t="n">
-        <v>2462.7</v>
+        <v>2471.8</v>
       </c>
     </row>
     <row r="68">
@@ -1654,7 +1654,7 @@
         <v>2716.3</v>
       </c>
       <c r="C68" t="n">
-        <v>2470.2</v>
+        <v>2479.6</v>
       </c>
     </row>
     <row r="69">
@@ -1667,7 +1667,7 @@
         <v>2555.7</v>
       </c>
       <c r="C69" t="n">
-        <v>2477.8</v>
+        <v>2487.5</v>
       </c>
     </row>
     <row r="70">
@@ -1680,7 +1680,7 @@
         <v>2489.4</v>
       </c>
       <c r="C70" t="n">
-        <v>2485.3</v>
+        <v>2495.3</v>
       </c>
     </row>
     <row r="71">
@@ -1693,7 +1693,7 @@
         <v>2585.2</v>
       </c>
       <c r="C71" t="n">
-        <v>2492.8</v>
+        <v>2503.1</v>
       </c>
     </row>
     <row r="72">
@@ -1706,7 +1706,7 @@
         <v>2403.3</v>
       </c>
       <c r="C72" t="n">
-        <v>2500.4</v>
+        <v>2510.9</v>
       </c>
     </row>
     <row r="73">
@@ -1719,7 +1719,7 @@
         <v>2513.7</v>
       </c>
       <c r="C73" t="n">
-        <v>2507.9</v>
+        <v>2518.7</v>
       </c>
     </row>
     <row r="74">
@@ -1732,7 +1732,7 @@
         <v>2615.5</v>
       </c>
       <c r="C74" t="n">
-        <v>2515.4</v>
+        <v>2526.6</v>
       </c>
     </row>
     <row r="75">
@@ -1745,7 +1745,7 @@
         <v>2487.6</v>
       </c>
       <c r="C75" t="n">
-        <v>2523</v>
+        <v>2534.4</v>
       </c>
     </row>
     <row r="76">
@@ -1758,7 +1758,7 @@
         <v>2757.3</v>
       </c>
       <c r="C76" t="n">
-        <v>2530.5</v>
+        <v>2542.2</v>
       </c>
     </row>
     <row r="77">
@@ -1771,7 +1771,7 @@
         <v>2556.3</v>
       </c>
       <c r="C77" t="n">
-        <v>2538</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="78">
@@ -1784,7 +1784,7 @@
         <v>2708.4</v>
       </c>
       <c r="C78" t="n">
-        <v>2545.5</v>
+        <v>2557.9</v>
       </c>
     </row>
     <row r="79">
@@ -1797,7 +1797,7 @@
         <v>2518.3</v>
       </c>
       <c r="C79" t="n">
-        <v>2553.1</v>
+        <v>2565.7</v>
       </c>
     </row>
     <row r="80">
@@ -1810,7 +1810,7 @@
         <v>2537</v>
       </c>
       <c r="C80" t="n">
-        <v>2560.6</v>
+        <v>2573.5</v>
       </c>
     </row>
     <row r="81">
@@ -1823,7 +1823,7 @@
         <v>2514.8</v>
       </c>
       <c r="C81" t="n">
-        <v>2568.1</v>
+        <v>2581.3</v>
       </c>
     </row>
     <row r="82">
@@ -1836,7 +1836,7 @@
         <v>2286.8</v>
       </c>
       <c r="C82" t="n">
-        <v>2575.7</v>
+        <v>2589.1</v>
       </c>
     </row>
     <row r="83">
@@ -1849,7 +1849,7 @@
         <v>1975.5</v>
       </c>
       <c r="C83" t="n">
-        <v>2583.2</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="84">
@@ -1862,7 +1862,7 @@
         <v>1853.5</v>
       </c>
       <c r="C84" t="n">
-        <v>2590.7</v>
+        <v>2604.8</v>
       </c>
     </row>
     <row r="85">
@@ -1875,7 +1875,7 @@
         <v>2355.2</v>
       </c>
       <c r="C85" t="n">
-        <v>2598.3</v>
+        <v>2612.6</v>
       </c>
     </row>
     <row r="86">
@@ -1888,7 +1888,7 @@
         <v>2604.6</v>
       </c>
       <c r="C86" t="n">
-        <v>2605.8</v>
+        <v>2620.4</v>
       </c>
     </row>
     <row r="87">
@@ -1901,7 +1901,7 @@
         <v>2566.3</v>
       </c>
       <c r="C87" t="n">
-        <v>2613.3</v>
+        <v>2628.3</v>
       </c>
     </row>
     <row r="88">
@@ -1914,7 +1914,7 @@
         <v>2849</v>
       </c>
       <c r="C88" t="n">
-        <v>2620.9</v>
+        <v>2636.1</v>
       </c>
     </row>
     <row r="89">
@@ -1927,7 +1927,7 @@
         <v>2774.5</v>
       </c>
       <c r="C89" t="n">
-        <v>2628.4</v>
+        <v>2643.9</v>
       </c>
     </row>
     <row r="90">
@@ -1940,7 +1940,7 @@
         <v>2794.3</v>
       </c>
       <c r="C90" t="n">
-        <v>2635.9</v>
+        <v>2651.7</v>
       </c>
     </row>
     <row r="91">
@@ -1953,7 +1953,7 @@
         <v>2573.7</v>
       </c>
       <c r="C91" t="n">
-        <v>2643.5</v>
+        <v>2659.6</v>
       </c>
     </row>
     <row r="92">
@@ -1966,7 +1966,7 @@
         <v>2605.6</v>
       </c>
       <c r="C92" t="n">
-        <v>2651</v>
+        <v>2667.4</v>
       </c>
     </row>
     <row r="93">
@@ -1979,7 +1979,7 @@
         <v>2592.2</v>
       </c>
       <c r="C93" t="n">
-        <v>2658.5</v>
+        <v>2675.2</v>
       </c>
     </row>
     <row r="94">
@@ -1992,7 +1992,7 @@
         <v>2667.9</v>
       </c>
       <c r="C94" t="n">
-        <v>2666.1</v>
+        <v>2683</v>
       </c>
     </row>
     <row r="95">
@@ -2005,7 +2005,7 @@
         <v>2802.6</v>
       </c>
       <c r="C95" t="n">
-        <v>2673.6</v>
+        <v>2690.8</v>
       </c>
     </row>
     <row r="96">
@@ -2018,7 +2018,7 @@
         <v>2696.6</v>
       </c>
       <c r="C96" t="n">
-        <v>2681.1</v>
+        <v>2698.7</v>
       </c>
     </row>
     <row r="97">
@@ -2031,7 +2031,7 @@
         <v>2828.5</v>
       </c>
       <c r="C97" t="n">
-        <v>2688.7</v>
+        <v>2706.5</v>
       </c>
     </row>
     <row r="98">
@@ -2044,7 +2044,7 @@
         <v>2685.6</v>
       </c>
       <c r="C98" t="n">
-        <v>2696.2</v>
+        <v>2714.3</v>
       </c>
     </row>
     <row r="99">
@@ -2057,7 +2057,7 @@
         <v>2609.1</v>
       </c>
       <c r="C99" t="n">
-        <v>2703.7</v>
+        <v>2722.1</v>
       </c>
     </row>
     <row r="100">
@@ -2070,7 +2070,7 @@
         <v>3010.2</v>
       </c>
       <c r="C100" t="n">
-        <v>2711.3</v>
+        <v>2730</v>
       </c>
     </row>
     <row r="101">
@@ -2083,7 +2083,7 @@
         <v>2911.6</v>
       </c>
       <c r="C101" t="n">
-        <v>2718.8</v>
+        <v>2737.8</v>
       </c>
     </row>
     <row r="102">
@@ -2096,7 +2096,7 @@
         <v>3074.6</v>
       </c>
       <c r="C102" t="n">
-        <v>2726.3</v>
+        <v>2745.6</v>
       </c>
     </row>
     <row r="103">
@@ -2106,10 +2106,23 @@
         </is>
       </c>
       <c r="B103" t="n">
-        <v>2985.4</v>
+        <v>3040.6</v>
       </c>
       <c r="C103" t="n">
-        <v>2733.9</v>
+        <v>2753.4</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Jul 2026</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>3205.9</v>
+      </c>
+      <c r="C104" t="n">
+        <v>2761.2</v>
       </c>
     </row>
   </sheetData>
@@ -2123,7 +2136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4402,6 +4415,50 @@
         <v>867.371383</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>151.91731</v>
+      </c>
+      <c r="C104" t="n">
+        <v>447.178229</v>
+      </c>
+      <c r="D104" t="n">
+        <v>659.1966640000001</v>
+      </c>
+      <c r="E104" t="n">
+        <v>281.745417</v>
+      </c>
+      <c r="F104" t="n">
+        <v>871.897195</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>17.928054</v>
+      </c>
+      <c r="C105" t="n">
+        <v>29.770021</v>
+      </c>
+      <c r="D105" t="n">
+        <v>44.383431</v>
+      </c>
+      <c r="E105" t="n">
+        <v>15.288094</v>
+      </c>
+      <c r="F105" t="n">
+        <v>64.80995799999999</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>